<commit_message>
sync: update page-copy workbooks, regenerate content, mobile responsive polish
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/page-copy/01-首页.xlsx
+++ b/docs/page-copy/01-首页.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12255"/>
+    <workbookView windowWidth="27360" windowHeight="15030"/>
   </bookViews>
   <sheets>
     <sheet name="copy" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="245">
   <si>
     <t>block_key</t>
   </si>
@@ -657,6 +657,9 @@
   </si>
   <si>
     <t>siteContent.home.introTitle</t>
+  </si>
+  <si>
+    <t>什么是ASRA</t>
   </si>
   <si>
     <t>common.classifiedFiles</t>
@@ -1765,7 +1768,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G81"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="36.8333333333333" customWidth="1"/>
     <col min="2" max="2" width="28.8333333333333" customWidth="1"/>
@@ -3330,7 +3333,7 @@
         <v>60</v>
       </c>
       <c r="E68" t="s">
-        <v>12</v>
+        <v>65</v>
       </c>
       <c r="F68" t="s">
         <v>12</v>
@@ -3353,7 +3356,7 @@
         <v>93</v>
       </c>
       <c r="E69" t="s">
-        <v>12</v>
+        <v>94</v>
       </c>
       <c r="F69" t="s">
         <v>12</v>
@@ -3376,7 +3379,7 @@
         <v>96</v>
       </c>
       <c r="E70" t="s">
-        <v>12</v>
+        <v>210</v>
       </c>
       <c r="F70" t="s">
         <v>12</v>
@@ -3387,19 +3390,19 @@
     </row>
     <row r="71" spans="1:7">
       <c r="A71" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B71" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C71" t="s">
         <v>9</v>
       </c>
       <c r="D71" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E71" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F71" t="s">
         <v>12</v>
@@ -3410,19 +3413,19 @@
     </row>
     <row r="72" spans="1:7">
       <c r="A72" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B72" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C72" t="s">
         <v>9</v>
       </c>
       <c r="D72" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E72" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F72" t="s">
         <v>12</v>
@@ -3433,19 +3436,19 @@
     </row>
     <row r="73" spans="1:7">
       <c r="A73" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B73" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C73" t="s">
         <v>9</v>
       </c>
       <c r="D73" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E73" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F73" t="s">
         <v>12</v>
@@ -3456,19 +3459,19 @@
     </row>
     <row r="74" spans="1:7">
       <c r="A74" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B74" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C74" t="s">
         <v>9</v>
       </c>
       <c r="D74" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E74" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="F74" t="s">
         <v>12</v>
@@ -3479,19 +3482,19 @@
     </row>
     <row r="75" spans="1:7">
       <c r="A75" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B75" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C75" t="s">
         <v>9</v>
       </c>
       <c r="D75" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E75" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F75" t="s">
         <v>12</v>
@@ -3502,19 +3505,19 @@
     </row>
     <row r="76" spans="1:7">
       <c r="A76" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B76" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C76" t="s">
         <v>9</v>
       </c>
       <c r="D76" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="E76" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F76" t="s">
         <v>12</v>
@@ -3525,19 +3528,19 @@
     </row>
     <row r="77" spans="1:7">
       <c r="A77" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B77" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C77" t="s">
         <v>9</v>
       </c>
       <c r="D77" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E77" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="F77" t="s">
         <v>12</v>
@@ -3548,19 +3551,19 @@
     </row>
     <row r="78" spans="1:7">
       <c r="A78" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B78" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C78" t="s">
         <v>9</v>
       </c>
       <c r="D78" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E78" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F78" t="s">
         <v>12</v>
@@ -3571,19 +3574,19 @@
     </row>
     <row r="79" spans="1:7">
       <c r="A79" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B79" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C79" t="s">
         <v>9</v>
       </c>
       <c r="D79" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E79" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F79" t="s">
         <v>12</v>
@@ -3594,19 +3597,19 @@
     </row>
     <row r="80" spans="1:7">
       <c r="A80" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B80" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C80" t="s">
         <v>9</v>
       </c>
       <c r="D80" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E80" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F80" t="s">
         <v>12</v>
@@ -3617,19 +3620,19 @@
     </row>
     <row r="81" spans="1:7">
       <c r="A81" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B81" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C81" t="s">
         <v>9</v>
       </c>
       <c r="D81" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E81" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F81" t="s">
         <v>12</v>
@@ -3642,7 +3645,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A71:G81 E69:G70 A69:C70 A55:D55 F54:G55 A56:G56 A57:D57 F57:G57 A58:G60 A61:D62 F61:G62 A63:G68 A54:C54 A49:G50 A51:D51 F51:G52 A52:C52 A53:G53 F48:G48 A48:C48 A47:G47 F46:G46 A46:C46 A37:G39 A40:D40 F40:G40 A41:G41 A42:D42 F42:G42 A43:G43 A44:D44 F44:G44 A45:G45 F35:G36 A35:C36 A32:G32 A33:D33 F33:G33 A34:G34 F29:G31 A29:C31 A26:D26 F25:G26 A27:G28 A25:C25 A23:G24 F21:G22 A22:C22 A20:G20 A21:D21 F18:G19 A19:C19 B18:C18 B16:D16 F15:G16 B17:G17 A13:G14 A15:D15 F10:G12 A10:C12 A2:C7 F5:G7 A8:G9 E2:G2 F3:G4 A1:G1" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:G1 E2:G2 A8:G9 F3:G7 A2:C7 A10:C12 F10:G12 A15:D15 A13:G14 B17:G17 F15:G16 B16:D16 B18:C18 A19:C19 F18:G19 A21:D21 A20:G20 A22:C22 F21:G22 A23:G24 A25:C25 A27:G28 F25:G26 A26:D26 A29:C31 F29:G31 A34:G34 F33:G33 A33:D33 A32:G32 A35:C36 F35:G36 A45:G45 F44:G44 A44:D44 A43:G43 F42:G42 A42:D42 A41:G41 F40:G40 A40:D40 A37:G39 A46:C46 F46:G46 A47:G47 A48:C48 F48:G48 A53:G53 A52:C52 F51:G52 A51:D51 A49:G50 A54:C54 A63:G67 A68:D68 F68:G70 F61:G62 A61:D62 A58:G60 F57:G57 A57:D57 A56:G56 F54:G55 A55:D55 A69:C70 A71:G81" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Flush EN overrides to xlsx; clear spiritTerminologyEnOverrides — editor now controls all EN copy
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/page-copy/01-首页.xlsx
+++ b/docs/page-copy/01-首页.xlsx
@@ -439,8 +439,8 @@
       <c r="D2" t="str" xml:space="preserve">
         <v xml:space="preserve">255+ recorded public welfare live broadcasts; 800+ broadcast hours; TikTok pushed to 70,000+ highly relevant visitors; 1,200+ in-depth interviews.
 Among them:
-In-depth communication with 400+ attached spirit ghosts.
-Helped 240+ patients with mental disorders quickly relieve the suffering caused by attached spirit ghosts on-site.</v>
+In-depth communication with 400+ attached **spirits (ghosts)**.
+Helped 240+ patients with mental disorders quickly relieve the suffering caused by attached **spirits (ghosts)** on-site.</v>
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">255+有记录的公益直播；800+ 播出小时； Tiktok推送70,000+高相关人士来访 ；1,200+人次深度访谈；
@@ -490,8 +490,8 @@
       </c>
       <c r="D4" t="str" xml:space="preserve">
         <v xml:space="preserve">The achievements in the live broadcast were filmed into the second season of the documentary 'Woos Spirit Medicine.'
-1. Statistics on the survival status of spirit ghosts in the United States.
-2. Especially interesting and valuable spirit ghost cases.
+1. Statistics on the survival status of **spirits (ghosts)** in the United States.
+2. Especially interesting and valuable **spirit (ghost)** cases.
 3. Cases of master spirit members of SMSC appearing in the live broadcast.
 4. Special cases in the spiritual realm, such as doctors and hospitals, and situations where cult members are specially attached.</v>
       </c>
@@ -635,7 +635,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D10" t="str">
-        <v>ASRA Founder Caros Woo will use PRCASG superpowers in 2025 to systematically communicate with the attached ghosts on American patients with mental disorders through TikTok live broadcasts, revealing the true living conditions of American ghosts, and quickly help patients in the live room improve various pains and disorders caused by the attached spirit ghosts.</v>
+        <v>ASRA Founder Caros Woo will use PRCASG superpowers in 2025 to systematically communicate with the **spirits (ghosts)** on American patients with mental disorders through TikTok live broadcasts, revealing the true living conditions of American **spirits (ghosts)**, and quickly help patients in the live room improve various pains and disorders caused by attached **spirits (ghosts)**.</v>
       </c>
       <c r="E10" t="str">
         <v>ASRA会长Caros Woo在2025年使用PRCASG超能力通过TikTok直播系统性的与美国精神障碍患者身上的附体鬼魂系统性的交流美国鬼魂的真实生存状态，并且在直播间快速帮助患者改善附体鬼魂带来的各种病痛和灾害</v>
@@ -1054,7 +1054,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D28" t="str">
-        <v>The spiritual world has various types of master spirits. Among them, some are specifically responsible for helping ASRA members acquire the PRCASG superpower to control ghosts; they are called controllers among the master spirits. The spiritual world has specifically established associations to train and coordinate tens of thousands of master spirits to become controllers, in order to effectively connect with and assist ASRA members</v>
+        <v>The spiritual world has various types of master spirits. Among them, some are specifically responsible for helping ASRA members acquire the PRCASG superpower to control **spirits (ghosts)**; they are called controllers among the master spirits. The spiritual world has specifically established associations to train and coordinate tens of thousands of master spirits to become controllers, in order to effectively connect with and assist ASRA members</v>
       </c>
       <c r="E28" t="str" xml:space="preserve">
         <v xml:space="preserve">灵魂世界有各种类型的高级掌控灵( Master spirit)。其中一部分专门负责帮助ASRA会员获得控制鬼魂的PRCASG超能力,他们被称为高级掌控灵中的控制者.
@@ -1287,7 +1287,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D38" t="str">
-        <v>As the founder of ASRA, Woos family filmed a series of three-season documentaries of Woos ethereal life and world for over 1,400 minutes. This documentary is the first time in human history to systematically explore and reveal the truth of spirit realm and governor with a large amount of evidence</v>
+        <v>As the founder of ASRA, Woos family filmed a series of three-season documentaries of Woos ethereal life and world for over 1,400 minutes. This documentary is the first time in human history to systematically explore and reveal the truth of **spirit (soul)**, life, world and governor with a large amount of evidence</v>
       </c>
       <c r="E38" t="str">
         <v>作为ASRA协会的会长和创始人，吴氏父子拍摄了超1400分钟《吴氏灵魂生命与世界》的3季系列纪录片。该纪录片是人类历史上第1次用大量的证据，系统性的探索和揭示了灵魂生命、世界和统御者的真相。</v>
@@ -1356,7 +1356,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D41" t="str">
-        <v>Collecting all true scientific research materials from East and West regarding spirits, PSI, NDE, past-life memories, and other topics related to spirits and the Ethereal Realm. With personal possession, supernatural and spirit-exorcism experiences.</v>
+        <v>Collecting all true scientific research materials from East and West regarding **spirit (soul)**, PSI, NDE, past-life memories, and other topics related to **spirit (soul)** and the Ethereal Realm. With personal possession, supernatural and spirit-exorcism experiences.</v>
       </c>
       <c r="E41" t="str">
         <v>汇集东西方关于灵体、超感知、濒死体验、前世记忆等与灵及灵魂世界相关的真实科研材料，附个人附体、灵异与驱灵经历。</v>
@@ -1448,7 +1448,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D45" t="str">
-        <v>This documentary provides the evidence of spirits and ghosts existing while people are alive and after death from scientific perspective and how it cause illness to the physical body. The organs, physiological systems, and basic pathology of spirits.It contains four parts: 1. Evidence of the existence of spirits ghosts and the general situation of their existence. 2. Physiology of human spirit soul 3. Pathology of human spirit soul 4. Physiology and pathology of spirits ghosts</v>
+        <v>This documentary provides, from a scientific perspective, evidence that **spirit** (the in-body **spirit**) and **spirits (ghosts)** exist both before and after death, and shows how they can cause illness in the physical body—the organs, physiological systems, and basic pathology involved. It contains four parts: (1) Evidence for **spirits (ghosts)** and their general situation. (2) Physiology of the human **spirit (soul)**. (3) Pathology of the human **spirit (soul)**. (4) Physiology and pathology of **spirits (ghosts)**.</v>
       </c>
       <c r="E45" t="str" xml:space="preserve">
         <v xml:space="preserve">从科学视角呈现鬼魂在人类生与死时存在的证据，及其如何致病于肉体：灵体的器官、生理系统与基本病理学。包含4个板块：
@@ -1544,7 +1544,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D49" t="str">
-        <v>The management authority of the master spirit is given by the superiors layer after layer. The ultimate superior is UMMA. The spiritual realm and our 13 billion-year-old real universe are not natural products, but are created by the creator --UMMA. His soul control system and team control the consciousness of human freedom, the evolution of life on earth and the ultimate fate of human civilization</v>
+        <v>The management authority of the master spirit is given by the superiors layer after layer. The ultimate superior is UMMA. The spiritual realm and our 13 billion-year-old real universe are not natural products, but are created by the creator --UMMA. His **spirit (soul)** control system and team control the consciousness of human freedom, the evolution of life on earth and the ultimate fate of human civilization</v>
       </c>
       <c r="E49" t="str">
         <v>高级掌控灵的管理权限是由一层又一层的上级给予的。这最终的上级就是 UMMA。灵魂世界和我们130亿年的现实宇宙并非天然产物，是由造物主--UMMA造就的。他的灵魂控制系统和队伍掌控着人类自由意识、地球生命的演化与人类文明的终极命运</v>

</xml_diff>

<commit_message>
Reorder spirit medicine outline: FILE 2-4 moved before FILE 2-3, FILE 2-5 stays last
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/page-copy/01-首页.xlsx
+++ b/docs/page-copy/01-首页.xlsx
@@ -635,7 +635,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D10" t="str">
-        <v>ASRA Founder Caros Woo will use PRCASG superpowers in 2025 to systematically communicate with the **spirits (ghosts)** on American patients with mental disorders through TikTok live broadcasts, revealing the true living conditions of American **spirits (ghosts)**, and quickly help patients in the live room improve various pains and disorders caused by attached **spirits (ghosts)**.</v>
+        <v>ASRA Founder Caros Woo used PRCASG superpowers in 2025 to systematically communicate with the **spirits (ghosts)** on American patients with mental disorders through TikTok live broadcasts, revealing the true living conditions of American **spirits (ghosts)**, and quickly help patients in the live room improve various diseases and disorders caused by attached **spirits (ghosts)**.</v>
       </c>
       <c r="E10" t="str">
         <v>ASRA会长Caros Woo在2025年使用PRCASG超能力通过TikTok直播系统性的与美国精神障碍患者身上的附体鬼魂系统性的交流美国鬼魂的真实生存状态，并且在直播间快速帮助患者改善附体鬼魂带来的各种病痛和灾害</v>
@@ -1287,7 +1287,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D38" t="str">
-        <v>As the founder of ASRA, Woos family filmed a series of three-season documentaries of Woos ethereal life and world for over 1,400 minutes. This documentary is the first time in human history to systematically explore and reveal the truth of **spirit (soul)**, life, world and governor with a large amount of evidence</v>
+        <v>As the founder of ASRA, Woos family filmed a series of three-season documentaries of spirit life and world for over 1,400 minutes. This documentary is the first time in human history to systematically explore and reveal the truth of **spirit **life, world and governor with a large amount of evidence</v>
       </c>
       <c r="E38" t="str">
         <v>作为ASRA协会的会长和创始人，吴氏父子拍摄了超1400分钟《吴氏灵魂生命与世界》的3季系列纪录片。该纪录片是人类历史上第1次用大量的证据，系统性的探索和揭示了灵魂生命、世界和统御者的真相。</v>
@@ -1447,8 +1447,12 @@
       <c r="C45" t="str">
         <v>paragraph / other</v>
       </c>
-      <c r="D45" t="str">
-        <v>This documentary provides, from a scientific perspective, evidence that **spirit** (the in-body **spirit**) and **spirits (ghosts)** exist both before and after death, and shows how they can cause illness in the physical body—the organs, physiological systems, and basic pathology involved. It contains four parts: (1) Evidence for **spirits (ghosts)** and their general situation. (2) Physiology of the human **spirit (soul)**. (3) Pathology of the human **spirit (soul)**. (4) Physiology and pathology of **spirits (ghosts)**.</v>
+      <c r="D45" t="str" xml:space="preserve">
+        <v xml:space="preserve">This documentary provides, from a scientific perspective, evidence that **spirit (soul**) and **spirits (ghosts)** exist both before and after death, and shows how they can cause illness in the physical body—the organs, physiological systems, and basic pathology involved. It contains four parts: 
+(1) Evidence for **spirits (ghosts)** and their general situation. 
+(2) Physiology of the human **spirit (soul)**. 
+(3) Pathology of the human **spirit (soul)**. 
+(4) Physiology and pathology of **spirits (ghosts)**.</v>
       </c>
       <c r="E45" t="str" xml:space="preserve">
         <v xml:space="preserve">从科学视角呈现鬼魂在人类生与死时存在的证据，及其如何致病于肉体：灵体的器官、生理系统与基本病理学。包含4个板块：
@@ -1544,7 +1548,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D49" t="str">
-        <v>The management authority of the master spirit is given by the superiors layer after layer. The ultimate superior is UMMA. The spiritual realm and our 13 billion-year-old real universe are not natural products, but are created by the creator --UMMA. His **spirit (soul)** control system and team control the consciousness of human freedom, the evolution of life on earth and the ultimate fate of human civilization</v>
+        <v>The management authority of the master spirit is given by the superiors layer after layer. The ultimate superior is UMMA. The spiritual realm and our 13 billion-year-old real universe are not natural products, but are created by the creator --UMMA. His **spirit (soul)** control system and team control the consciousness of human free will, the evolution of life on earth and the ultimate fate of human civilization</v>
       </c>
       <c r="E49" t="str">
         <v>高级掌控灵的管理权限是由一层又一层的上级给予的。这最终的上级就是 UMMA。灵魂世界和我们130亿年的现实宇宙并非天然产物，是由造物主--UMMA造就的。他的灵魂控制系统和队伍掌控着人类自由意识、地球生命的演化与人类文明的终极命运</v>

</xml_diff>